<commit_message>
chore: Some pre-processing for credit table matcher
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/Fichier de configuration GRAAL - Test integrations.xlsx
+++ b/tests/integration/test_data/Fichier de configuration GRAAL - Test integrations.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C7DB789-95B7-724C-A485-307EEAA8B036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{675CF26D-6392-8546-A88D-17FB780F10B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Code et Article" sheetId="1" r:id="rId1"/>
     <sheet name="Mots clés" sheetId="2" r:id="rId2"/>
-    <sheet name="Prénom Nom Mail" sheetId="3" r:id="rId3"/>
+    <sheet name="Infos Agents" sheetId="3" r:id="rId3"/>
     <sheet name="Attribution par défaut" sheetId="4" r:id="rId4"/>
     <sheet name="Acronymes" sheetId="5" r:id="rId5"/>
   </sheets>
@@ -1220,7 +1220,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1292,10 +1292,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -31011,101 +31010,101 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A2" s="29" t="s">
+      <c r="A2" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="C2" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A4" s="29" t="s">
+      <c r="A4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A5" s="29" t="s">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A6" s="29" t="s">
+      <c r="A6" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A9" s="29" t="s">
+      <c r="A9" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A10" s="29" t="s">
+      <c r="A10" t="s">
         <v>342</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="31" t="s">
         <v>344</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C10" t="s">
         <v>345</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat (attribution): Handle plurals
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/Fichier de configuration GRAAL - Test integrations.xlsx
+++ b/tests/integration/test_data/Fichier de configuration GRAAL - Test integrations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{675CF26D-6392-8546-A88D-17FB780F10B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40DA162F-CF50-0B48-9B44-ECB4055C0575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Code et Article" sheetId="1" r:id="rId1"/>
@@ -220,9 +220,6 @@
     <t>montant Z</t>
   </si>
   <si>
-    <t>charges patronales</t>
-  </si>
-  <si>
     <t>composantes salariales</t>
   </si>
   <si>
@@ -1070,6 +1067,9 @@
   </si>
   <si>
     <t>CABC</t>
+  </si>
+  <si>
+    <t>charge patronale</t>
   </si>
 </sst>
 </file>
@@ -3168,7 +3168,7 @@
     </row>
     <row r="8" spans="1:26" ht="15.75" customHeight="1">
       <c r="A8" s="16" t="s">
-        <v>62</v>
+        <v>345</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>15</v>
@@ -3200,7 +3200,7 @@
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1">
       <c r="A9" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>6</v>
@@ -3232,10 +3232,10 @@
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1">
       <c r="A10" s="26" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="13"/>
@@ -31003,10 +31003,10 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C1" s="28" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" customHeight="1">
@@ -31014,10 +31014,10 @@
         <v>19</v>
       </c>
       <c r="B2" s="29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" customHeight="1">
@@ -31025,10 +31025,10 @@
         <v>15</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C3" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.75" customHeight="1">
@@ -31036,10 +31036,10 @@
         <v>21</v>
       </c>
       <c r="B4" s="29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15.75" customHeight="1">
@@ -31047,10 +31047,10 @@
         <v>6</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15.75" customHeight="1">
@@ -31058,32 +31058,32 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15.75" customHeight="1">
       <c r="A7" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="29" t="s">
-        <v>71</v>
-      </c>
       <c r="C7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15.75" customHeight="1">
       <c r="A8" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="29" t="s">
-        <v>73</v>
-      </c>
       <c r="C8" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.75" customHeight="1">
@@ -31091,21 +31091,21 @@
         <v>60</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" customHeight="1">
       <c r="A10" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B10" s="31" t="s">
+        <v>343</v>
+      </c>
+      <c r="C10" t="s">
         <v>344</v>
-      </c>
-      <c r="C10" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.75" customHeight="1"/>
@@ -32129,7 +32129,7 @@
     </row>
     <row r="2" spans="1:1" ht="15.75" customHeight="1">
       <c r="A2" s="21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.75" customHeight="1">
@@ -33149,1050 +33149,1050 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>75</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="24" t="s">
         <v>77</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="24" t="s">
         <v>79</v>
-      </c>
-      <c r="B3" s="24" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="24" t="s">
         <v>81</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="24" t="s">
         <v>83</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" s="24" t="s">
         <v>85</v>
-      </c>
-      <c r="B6" s="24" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="24" t="s">
         <v>87</v>
-      </c>
-      <c r="B7" s="24" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="24" t="s">
         <v>89</v>
-      </c>
-      <c r="B8" s="24" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="24" t="s">
         <v>91</v>
-      </c>
-      <c r="B9" s="24" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="24" t="s">
         <v>93</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="24" t="s">
         <v>95</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="24" t="s">
         <v>97</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="24" t="s">
         <v>99</v>
-      </c>
-      <c r="B13" s="24" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" s="24" t="s">
         <v>101</v>
-      </c>
-      <c r="B14" s="24" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="B15" s="24" t="s">
         <v>103</v>
-      </c>
-      <c r="B15" s="24" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="B16" s="24" t="s">
         <v>105</v>
-      </c>
-      <c r="B16" s="24" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" s="24" t="s">
         <v>107</v>
-      </c>
-      <c r="B17" s="24" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" s="24" t="s">
         <v>109</v>
-      </c>
-      <c r="B18" s="24" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="B19" s="24" t="s">
         <v>111</v>
-      </c>
-      <c r="B19" s="24" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="B20" s="24" t="s">
         <v>113</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B21" s="24" t="s">
         <v>115</v>
-      </c>
-      <c r="B21" s="24" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="B22" s="24" t="s">
         <v>117</v>
-      </c>
-      <c r="B22" s="24" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="B23" s="24" t="s">
         <v>119</v>
-      </c>
-      <c r="B23" s="24" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" s="24" t="s">
         <v>121</v>
-      </c>
-      <c r="B24" s="24" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" s="24" t="s">
         <v>123</v>
-      </c>
-      <c r="B25" s="24" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="B26" s="24" t="s">
         <v>125</v>
-      </c>
-      <c r="B26" s="24" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="B27" s="24" t="s">
         <v>127</v>
-      </c>
-      <c r="B27" s="24" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="B28" s="24" t="s">
         <v>129</v>
-      </c>
-      <c r="B28" s="24" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="B29" s="24" t="s">
         <v>131</v>
-      </c>
-      <c r="B29" s="24" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="B30" s="24" t="s">
         <v>133</v>
-      </c>
-      <c r="B30" s="24" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="B31" s="24" t="s">
         <v>135</v>
-      </c>
-      <c r="B31" s="24" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="B32" s="24" t="s">
         <v>137</v>
-      </c>
-      <c r="B32" s="24" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="B33" s="24" t="s">
         <v>139</v>
-      </c>
-      <c r="B33" s="24" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="B34" s="24" t="s">
         <v>141</v>
-      </c>
-      <c r="B34" s="24" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="B35" s="24" t="s">
         <v>143</v>
-      </c>
-      <c r="B35" s="24" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="B36" s="24" t="s">
         <v>145</v>
-      </c>
-      <c r="B36" s="24" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="B37" s="24" t="s">
         <v>147</v>
-      </c>
-      <c r="B37" s="24" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="B38" s="24" t="s">
         <v>149</v>
-      </c>
-      <c r="B38" s="24" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="24" t="s">
+        <v>150</v>
+      </c>
+      <c r="B39" s="24" t="s">
         <v>151</v>
-      </c>
-      <c r="B39" s="24" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="B40" s="24" t="s">
         <v>153</v>
-      </c>
-      <c r="B40" s="24" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="25" t="s">
+        <v>154</v>
+      </c>
+      <c r="B41" s="24" t="s">
         <v>155</v>
-      </c>
-      <c r="B41" s="24" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="B42" s="24" t="s">
         <v>157</v>
-      </c>
-      <c r="B42" s="24" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="B43" s="24" t="s">
         <v>159</v>
-      </c>
-      <c r="B43" s="24" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="B44" s="24" t="s">
         <v>161</v>
-      </c>
-      <c r="B44" s="24" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="24" t="s">
+        <v>162</v>
+      </c>
+      <c r="B45" s="24" t="s">
         <v>163</v>
-      </c>
-      <c r="B45" s="24" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="24" t="s">
+        <v>164</v>
+      </c>
+      <c r="B46" s="24" t="s">
         <v>165</v>
-      </c>
-      <c r="B46" s="24" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="B47" s="24" t="s">
         <v>167</v>
-      </c>
-      <c r="B47" s="24" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="24" t="s">
+        <v>168</v>
+      </c>
+      <c r="B48" s="24" t="s">
         <v>169</v>
-      </c>
-      <c r="B48" s="24" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="24" t="s">
+        <v>170</v>
+      </c>
+      <c r="B49" s="24" t="s">
         <v>171</v>
-      </c>
-      <c r="B49" s="24" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="24" t="s">
+        <v>172</v>
+      </c>
+      <c r="B50" s="24" t="s">
         <v>173</v>
-      </c>
-      <c r="B50" s="24" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="24" t="s">
+        <v>174</v>
+      </c>
+      <c r="B51" s="24" t="s">
         <v>175</v>
-      </c>
-      <c r="B51" s="24" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="B52" s="24" t="s">
         <v>177</v>
-      </c>
-      <c r="B52" s="24" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="24" t="s">
+        <v>178</v>
+      </c>
+      <c r="B53" s="24" t="s">
         <v>179</v>
-      </c>
-      <c r="B53" s="24" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="24" t="s">
+        <v>180</v>
+      </c>
+      <c r="B54" s="24" t="s">
         <v>181</v>
-      </c>
-      <c r="B54" s="24" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="B55" s="24" t="s">
         <v>183</v>
-      </c>
-      <c r="B55" s="24" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="24" t="s">
+        <v>184</v>
+      </c>
+      <c r="B56" s="24" t="s">
         <v>185</v>
-      </c>
-      <c r="B56" s="24" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="B57" s="24" t="s">
         <v>187</v>
-      </c>
-      <c r="B57" s="24" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="B58" s="24" t="s">
         <v>189</v>
-      </c>
-      <c r="B58" s="24" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="24" t="s">
+        <v>190</v>
+      </c>
+      <c r="B59" s="24" t="s">
         <v>191</v>
-      </c>
-      <c r="B59" s="24" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="24" t="s">
+        <v>192</v>
+      </c>
+      <c r="B60" s="24" t="s">
         <v>193</v>
-      </c>
-      <c r="B60" s="24" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="B61" s="24" t="s">
         <v>195</v>
-      </c>
-      <c r="B61" s="24" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="24" t="s">
+        <v>196</v>
+      </c>
+      <c r="B62" s="24" t="s">
         <v>197</v>
-      </c>
-      <c r="B62" s="24" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="24" t="s">
+        <v>198</v>
+      </c>
+      <c r="B63" s="24" t="s">
         <v>199</v>
-      </c>
-      <c r="B63" s="24" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="24" t="s">
+        <v>200</v>
+      </c>
+      <c r="B64" s="24" t="s">
         <v>201</v>
-      </c>
-      <c r="B64" s="24" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="24" t="s">
+        <v>202</v>
+      </c>
+      <c r="B65" s="24" t="s">
         <v>203</v>
-      </c>
-      <c r="B65" s="24" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="24" t="s">
+        <v>204</v>
+      </c>
+      <c r="B66" s="24" t="s">
         <v>205</v>
-      </c>
-      <c r="B66" s="24" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="B67" s="24" t="s">
         <v>207</v>
-      </c>
-      <c r="B67" s="24" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="24" t="s">
+        <v>208</v>
+      </c>
+      <c r="B68" s="24" t="s">
         <v>209</v>
-      </c>
-      <c r="B68" s="24" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B69" s="24" t="s">
         <v>211</v>
-      </c>
-      <c r="B69" s="24" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="24" t="s">
+        <v>212</v>
+      </c>
+      <c r="B70" s="24" t="s">
         <v>213</v>
-      </c>
-      <c r="B70" s="24" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="24" t="s">
+        <v>214</v>
+      </c>
+      <c r="B71" s="24" t="s">
         <v>215</v>
-      </c>
-      <c r="B71" s="24" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="24" t="s">
+        <v>216</v>
+      </c>
+      <c r="B72" s="24" t="s">
         <v>217</v>
-      </c>
-      <c r="B72" s="24" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="24" t="s">
+        <v>218</v>
+      </c>
+      <c r="B73" s="24" t="s">
         <v>219</v>
-      </c>
-      <c r="B73" s="24" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="B74" s="24" t="s">
         <v>221</v>
-      </c>
-      <c r="B74" s="24" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="24" t="s">
+        <v>222</v>
+      </c>
+      <c r="B75" s="24" t="s">
         <v>223</v>
-      </c>
-      <c r="B75" s="24" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="24" t="s">
+        <v>224</v>
+      </c>
+      <c r="B76" s="24" t="s">
         <v>225</v>
-      </c>
-      <c r="B76" s="24" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="B77" s="24" t="s">
         <v>227</v>
-      </c>
-      <c r="B77" s="24" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="B78" s="24" t="s">
         <v>229</v>
-      </c>
-      <c r="B78" s="24" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="24" t="s">
+        <v>230</v>
+      </c>
+      <c r="B79" s="24" t="s">
         <v>231</v>
-      </c>
-      <c r="B79" s="24" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="24" t="s">
+        <v>232</v>
+      </c>
+      <c r="B80" s="24" t="s">
         <v>233</v>
-      </c>
-      <c r="B80" s="24" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="24" t="s">
+        <v>234</v>
+      </c>
+      <c r="B81" s="24" t="s">
         <v>235</v>
-      </c>
-      <c r="B81" s="24" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="24" t="s">
+        <v>236</v>
+      </c>
+      <c r="B82" s="24" t="s">
         <v>237</v>
-      </c>
-      <c r="B82" s="24" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="24" t="s">
+        <v>238</v>
+      </c>
+      <c r="B83" s="24" t="s">
         <v>239</v>
-      </c>
-      <c r="B83" s="24" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="24" t="s">
+        <v>240</v>
+      </c>
+      <c r="B84" s="24" t="s">
         <v>241</v>
-      </c>
-      <c r="B84" s="24" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="24" t="s">
+        <v>242</v>
+      </c>
+      <c r="B85" s="24" t="s">
         <v>243</v>
-      </c>
-      <c r="B85" s="24" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="24" t="s">
+        <v>244</v>
+      </c>
+      <c r="B86" s="24" t="s">
         <v>245</v>
-      </c>
-      <c r="B86" s="24" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="24" t="s">
+        <v>246</v>
+      </c>
+      <c r="B87" s="24" t="s">
         <v>247</v>
-      </c>
-      <c r="B87" s="24" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="B88" s="24" t="s">
         <v>249</v>
-      </c>
-      <c r="B88" s="24" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="24" t="s">
+        <v>250</v>
+      </c>
+      <c r="B89" s="24" t="s">
         <v>251</v>
-      </c>
-      <c r="B89" s="24" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="24" t="s">
+        <v>252</v>
+      </c>
+      <c r="B90" s="24" t="s">
         <v>253</v>
-      </c>
-      <c r="B90" s="24" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="24" t="s">
+        <v>254</v>
+      </c>
+      <c r="B91" s="24" t="s">
         <v>255</v>
-      </c>
-      <c r="B91" s="24" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="B92" s="24" t="s">
         <v>257</v>
-      </c>
-      <c r="B92" s="24" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="24" t="s">
+        <v>258</v>
+      </c>
+      <c r="B93" s="24" t="s">
         <v>259</v>
-      </c>
-      <c r="B93" s="24" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="24" t="s">
+        <v>260</v>
+      </c>
+      <c r="B94" s="24" t="s">
         <v>261</v>
-      </c>
-      <c r="B94" s="24" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="24" t="s">
+        <v>262</v>
+      </c>
+      <c r="B95" s="24" t="s">
         <v>263</v>
-      </c>
-      <c r="B95" s="24" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="24" t="s">
+        <v>264</v>
+      </c>
+      <c r="B96" s="24" t="s">
         <v>265</v>
-      </c>
-      <c r="B96" s="24" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="24" t="s">
+        <v>266</v>
+      </c>
+      <c r="B97" s="24" t="s">
         <v>267</v>
-      </c>
-      <c r="B97" s="24" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="24" t="s">
+        <v>268</v>
+      </c>
+      <c r="B98" s="24" t="s">
         <v>269</v>
-      </c>
-      <c r="B98" s="24" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="24" t="s">
+        <v>270</v>
+      </c>
+      <c r="B99" s="24" t="s">
         <v>271</v>
-      </c>
-      <c r="B99" s="24" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="24" t="s">
+        <v>272</v>
+      </c>
+      <c r="B100" s="24" t="s">
         <v>273</v>
-      </c>
-      <c r="B100" s="24" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="24" t="s">
+        <v>274</v>
+      </c>
+      <c r="B101" s="24" t="s">
         <v>275</v>
-      </c>
-      <c r="B101" s="24" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="24" t="s">
+        <v>276</v>
+      </c>
+      <c r="B102" s="24" t="s">
         <v>277</v>
-      </c>
-      <c r="B102" s="24" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="24" t="s">
+        <v>278</v>
+      </c>
+      <c r="B103" s="24" t="s">
         <v>279</v>
-      </c>
-      <c r="B103" s="24" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="24" t="s">
+        <v>280</v>
+      </c>
+      <c r="B104" s="24" t="s">
         <v>281</v>
-      </c>
-      <c r="B104" s="24" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="24" t="s">
+        <v>282</v>
+      </c>
+      <c r="B105" s="24" t="s">
         <v>283</v>
-      </c>
-      <c r="B105" s="24" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="24" t="s">
+        <v>284</v>
+      </c>
+      <c r="B106" s="24" t="s">
         <v>285</v>
-      </c>
-      <c r="B106" s="24" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="24" t="s">
+        <v>286</v>
+      </c>
+      <c r="B107" s="24" t="s">
         <v>287</v>
-      </c>
-      <c r="B107" s="24" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="B108" s="24" t="s">
         <v>289</v>
-      </c>
-      <c r="B108" s="24" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="24" t="s">
+        <v>290</v>
+      </c>
+      <c r="B109" s="24" t="s">
         <v>291</v>
-      </c>
-      <c r="B109" s="24" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="24" t="s">
+        <v>292</v>
+      </c>
+      <c r="B110" s="24" t="s">
         <v>293</v>
-      </c>
-      <c r="B110" s="24" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="24" t="s">
+        <v>294</v>
+      </c>
+      <c r="B111" s="24" t="s">
         <v>295</v>
-      </c>
-      <c r="B111" s="24" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="24" t="s">
+        <v>296</v>
+      </c>
+      <c r="B112" s="24" t="s">
         <v>297</v>
-      </c>
-      <c r="B112" s="24" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="24" t="s">
+        <v>298</v>
+      </c>
+      <c r="B113" s="24" t="s">
         <v>299</v>
-      </c>
-      <c r="B113" s="24" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="24" t="s">
+        <v>300</v>
+      </c>
+      <c r="B114" s="24" t="s">
         <v>301</v>
-      </c>
-      <c r="B114" s="24" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" s="24" t="s">
+        <v>302</v>
+      </c>
+      <c r="B115" s="24" t="s">
         <v>303</v>
-      </c>
-      <c r="B115" s="24" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="24" t="s">
+        <v>304</v>
+      </c>
+      <c r="B116" s="24" t="s">
         <v>305</v>
-      </c>
-      <c r="B116" s="24" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="24" t="s">
+        <v>306</v>
+      </c>
+      <c r="B117" s="24" t="s">
         <v>307</v>
-      </c>
-      <c r="B117" s="24" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="24" t="s">
+        <v>308</v>
+      </c>
+      <c r="B118" s="24" t="s">
         <v>309</v>
-      </c>
-      <c r="B118" s="24" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="24" t="s">
+        <v>310</v>
+      </c>
+      <c r="B119" s="24" t="s">
         <v>311</v>
-      </c>
-      <c r="B119" s="24" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="24" t="s">
+        <v>312</v>
+      </c>
+      <c r="B120" s="24" t="s">
         <v>313</v>
-      </c>
-      <c r="B120" s="24" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="24" t="s">
+        <v>314</v>
+      </c>
+      <c r="B121" s="24" t="s">
         <v>315</v>
-      </c>
-      <c r="B121" s="24" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="24" t="s">
+        <v>316</v>
+      </c>
+      <c r="B122" s="24" t="s">
         <v>317</v>
-      </c>
-      <c r="B122" s="24" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="24" t="s">
+        <v>318</v>
+      </c>
+      <c r="B123" s="24" t="s">
         <v>319</v>
-      </c>
-      <c r="B123" s="24" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="24" t="s">
+        <v>320</v>
+      </c>
+      <c r="B124" s="24" t="s">
         <v>321</v>
-      </c>
-      <c r="B124" s="24" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="24" t="s">
+        <v>322</v>
+      </c>
+      <c r="B125" s="24" t="s">
         <v>323</v>
-      </c>
-      <c r="B125" s="24" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" s="24" t="s">
+        <v>324</v>
+      </c>
+      <c r="B126" s="24" t="s">
         <v>325</v>
-      </c>
-      <c r="B126" s="24" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="24" t="s">
+        <v>326</v>
+      </c>
+      <c r="B127" s="24" t="s">
         <v>327</v>
-      </c>
-      <c r="B127" s="24" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="24" t="s">
+        <v>328</v>
+      </c>
+      <c r="B128" s="24" t="s">
         <v>329</v>
-      </c>
-      <c r="B128" s="24" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="24" t="s">
+        <v>330</v>
+      </c>
+      <c r="B129" s="24" t="s">
         <v>331</v>
-      </c>
-      <c r="B129" s="24" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" s="24" t="s">
+        <v>332</v>
+      </c>
+      <c r="B130" s="24" t="s">
         <v>333</v>
-      </c>
-      <c r="B130" s="24" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="24" t="s">
+        <v>334</v>
+      </c>
+      <c r="B131" s="24" t="s">
         <v>335</v>
-      </c>
-      <c r="B131" s="24" t="s">
-        <v>336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>